<commit_message>
SPM-69: Release needs a reason; a released line can be asked for again
Releasing a reservation now needs a reason (up to 500 characters). It is
saved as Technical Support's notes and sent in the Coordinator's
notification, and reserving the line again clears it. When the Coordinator
changes the quantity of a released line, it goes back to Technical Support
as a fresh request. Changing only its technical requirements leaves it
released.

Tests written first. Manual cases SPM-69-TC01 to TC03 updated or added;
the workbook had not been run yet, so it was rebuilt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-69_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-69_Test_Cases.xlsx
@@ -18,6 +18,7 @@
     <sheet name="TC08" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="TC09" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="TC10" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="TC11" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -457,7 +458,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I26"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -550,7 +551,7 @@
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Technical Support releases a reservation after first cancelling, the line is marked Released, and its units become available to an overlapping event</t>
+          <t>Technical Support releases a reservation with a reason after first cancelling, the line is marked Released, and its units become available to an overlapping event</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
@@ -589,7 +590,7 @@
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>The assigned Coordinator is notified of the release, and the released reservation stays on the event's Equipment tab marked Released</t>
+          <t>The assigned Coordinator is notified of the release and its reason, and the released reservation stays on the event's Equipment tab marked Released</t>
         </is>
       </c>
       <c r="D5" s="11" t="inlineStr">
@@ -628,12 +629,12 @@
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>Technical Support reduces a reservation, the line becomes Partially fulfilled, the freed units show as available to an overlapping event, and the Coordinator is notified</t>
+          <t>Changing the quantity of a released line sends it back to Technical Support as a fresh request, while changing only its technical requirements leaves it released</t>
         </is>
       </c>
       <c r="D6" s="11" t="inlineStr">
         <is>
-          <t>AC2, AC4, AC5, AC6</t>
+          <t>AC7</t>
         </is>
       </c>
       <c r="E6" s="11" t="inlineStr">
@@ -643,7 +644,7 @@
       </c>
       <c r="F6" s="11" t="inlineStr">
         <is>
-          <t>Acceptance Criteria</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="G6" s="11" t="inlineStr">
@@ -667,17 +668,17 @@
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>An increase to one more unit than is available for the event's dates is refused and nothing is saved</t>
+          <t>Technical Support reduces a reservation, the line becomes Partially fulfilled, the freed units show as available to an overlapping event, and the Coordinator is notified</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>AC3</t>
+          <t>AC2, AC4, AC5, AC6</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>Boundary</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="F7" s="11" t="inlineStr">
@@ -706,22 +707,22 @@
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>The Adjust form refuses more than was requested, zero, and the quantity already reserved, and Cancel saves nothing</t>
+          <t>An increase to one more unit than is available for the event's dates is refused and nothing is saved</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>AC2, AC3</t>
+          <t>AC3</t>
         </is>
       </c>
       <c r="E8" s="11" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="F8" s="11" t="inlineStr">
         <is>
-          <t>Code</t>
+          <t>Acceptance Criteria</t>
         </is>
       </c>
       <c r="G8" s="11" t="inlineStr">
@@ -745,22 +746,22 @@
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Technical Support increases a reservation to exactly what is available, and the Coordinator is notified</t>
+          <t>The Adjust form refuses more than was requested, zero, and the quantity already reserved, and Cancel saves nothing</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>AC3, AC5, AC6</t>
+          <t>AC2, AC3</t>
         </is>
       </c>
       <c r="E9" s="11" t="inlineStr">
         <is>
-          <t>Boundary</t>
+          <t>Negative</t>
         </is>
       </c>
       <c r="F9" s="11" t="inlineStr">
         <is>
-          <t>Acceptance Criteria</t>
+          <t>Code</t>
         </is>
       </c>
       <c r="G9" s="11" t="inlineStr">
@@ -784,17 +785,17 @@
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>A Coordinator's change to a reserved requirement sends it back to Technical Support as Requested, still showing what is reserved, without flagging it</t>
+          <t>Technical Support increases a reservation to exactly what is available, and the Coordinator is notified</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>AC7</t>
+          <t>AC3, AC5, AC6</t>
         </is>
       </c>
       <c r="E10" s="11" t="inlineStr">
         <is>
-          <t>Positive</t>
+          <t>Boundary</t>
         </is>
       </c>
       <c r="F10" s="11" t="inlineStr">
@@ -823,12 +824,12 @@
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>Technical Support reviews a sent-back requirement and adjusts the reservation to the new quantity, marking it Reserved again</t>
+          <t>A Coordinator's change to a reserved requirement sends it back to Technical Support as Requested, still showing what is reserved, without flagging it</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>AC7, AC3, AC5</t>
+          <t>AC7</t>
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr">
@@ -862,17 +863,17 @@
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Adjust and Release are not offered on a line with nothing reserved, nor on a confirmed event</t>
+          <t>Technical Support reviews a sent-back requirement and adjusts the reservation to the new quantity, marking it Reserved again</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>AC1, AC2, AC3</t>
+          <t>AC7, AC3, AC5</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>Negative</t>
+          <t>Positive</t>
         </is>
       </c>
       <c r="F12" s="11" t="inlineStr">
@@ -901,7 +902,7 @@
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>The Event Coordinator cannot release or adjust a reservation, even by typing the Equipment request page's address</t>
+          <t>Adjust and Release are not offered on a line with nothing reserved, nor on a confirmed event</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
@@ -927,80 +928,96 @@
       <c r="H13" s="11" t="n"/>
       <c r="I13" s="11" t="n"/>
     </row>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>TC11</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>SPM-69-TC11</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>The Event Coordinator cannot release or adjust a reservation, even by typing the Equipment request page's address</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>AC1, AC2, AC3</t>
+        </is>
+      </c>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>Acceptance Criteria</t>
+        </is>
+      </c>
+      <c r="G14" s="11" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="H14" s="11" t="n"/>
+      <c r="I14" s="11" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>AC</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>Acceptance Criterion</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="n"/>
-      <c r="D16" s="9" t="n"/>
-      <c r="E16" s="7" t="inlineStr">
-        <is>
-          <t>Covered by</t>
-        </is>
-      </c>
-      <c r="F16" s="9" t="n"/>
-    </row>
-    <row r="17" ht="44.5" customHeight="1">
-      <c r="A17" s="11" t="inlineStr">
-        <is>
-          <t>AC1</t>
-        </is>
-      </c>
-      <c r="B17" s="11" t="inlineStr">
-        <is>
-          <t>Technical Support Staff can release an equipment reservation for an event.</t>
         </is>
       </c>
       <c r="C17" s="8" t="n"/>
       <c r="D17" s="9" t="n"/>
-      <c r="E17" s="11" t="inlineStr">
-        <is>
-          <t>SPM-69-TC01
-SPM-69-TC09
-SPM-69-TC10</t>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>Covered by</t>
         </is>
       </c>
       <c r="F17" s="9" t="n"/>
     </row>
-    <row r="18" ht="58" customHeight="1">
+    <row r="18" ht="44.5" customHeight="1">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>AC2</t>
+          <t>AC1</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>Technical Support Staff can reduce the reserved quantity of a reservation.</t>
+          <t>Technical Support Staff can release an equipment reservation for an event.</t>
         </is>
       </c>
       <c r="C18" s="8" t="n"/>
       <c r="D18" s="9" t="n"/>
       <c r="E18" s="11" t="inlineStr">
         <is>
-          <t>SPM-69-TC03
-SPM-69-TC05
-SPM-69-TC09
-SPM-69-TC10</t>
+          <t>SPM-69-TC01
+SPM-69-TC10
+SPM-69-TC11</t>
         </is>
       </c>
       <c r="F18" s="9" t="n"/>
     </row>
-    <row r="19" ht="85" customHeight="1">
+    <row r="19" ht="58" customHeight="1">
       <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>AC3</t>
+          <t>AC2</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>Technical Support Staff can increase the reserved quantity, and the system prevents an increase beyond the quantity available for the event's dates.</t>
+          <t>Technical Support Staff can reduce the reserved quantity of a reservation.</t>
         </is>
       </c>
       <c r="C19" s="8" t="n"/>
@@ -1008,45 +1025,47 @@
       <c r="E19" s="11" t="inlineStr">
         <is>
           <t>SPM-69-TC04
-SPM-69-TC05
 SPM-69-TC06
-SPM-69-TC08
-SPM-69-TC09
-SPM-69-TC10</t>
+SPM-69-TC10
+SPM-69-TC11</t>
         </is>
       </c>
       <c r="F19" s="9" t="n"/>
     </row>
-    <row r="20" ht="31" customHeight="1">
+    <row r="20" ht="85" customHeight="1">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>AC4</t>
+          <t>AC3</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>Given a reservation is released or reduced, when availability is next checked, then the freed quantity is available for overlapping events.</t>
+          <t>Technical Support Staff can increase the reserved quantity, and the system prevents an increase beyond the quantity available for the event's dates.</t>
         </is>
       </c>
       <c r="C20" s="8" t="n"/>
       <c r="D20" s="9" t="n"/>
       <c r="E20" s="11" t="inlineStr">
         <is>
-          <t>SPM-69-TC01
-SPM-69-TC03</t>
+          <t>SPM-69-TC05
+SPM-69-TC06
+SPM-69-TC07
+SPM-69-TC09
+SPM-69-TC10
+SPM-69-TC11</t>
         </is>
       </c>
       <c r="F20" s="9" t="n"/>
     </row>
-    <row r="21" ht="58" customHeight="1">
+    <row r="21" ht="31" customHeight="1">
       <c r="A21" s="11" t="inlineStr">
         <is>
-          <t>AC5</t>
+          <t>AC4</t>
         </is>
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>The fulfilment status of the related equipment requirement is updated to reflect the change (see: Review and Update Equipment Request).</t>
+          <t>Given a reservation is released or reduced, when availability is next checked, then the freed quantity is available for overlapping events.</t>
         </is>
       </c>
       <c r="C21" s="8" t="n"/>
@@ -1054,84 +1073,106 @@
       <c r="E21" s="11" t="inlineStr">
         <is>
           <t>SPM-69-TC01
-SPM-69-TC03
-SPM-69-TC06
-SPM-69-TC08</t>
+SPM-69-TC04</t>
         </is>
       </c>
       <c r="F21" s="9" t="n"/>
     </row>
-    <row r="22" ht="44.5" customHeight="1">
+    <row r="22" ht="58" customHeight="1">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>AC6</t>
+          <t>AC5</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>The assigned Event Coordinator is notified when a reservation for their event is released or adjusted.</t>
+          <t>The fulfilment status of the related equipment requirement is updated to reflect the change (see: Review and Update Equipment Request).</t>
         </is>
       </c>
       <c r="C22" s="8" t="n"/>
       <c r="D22" s="9" t="n"/>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>SPM-69-TC02
-SPM-69-TC03
-SPM-69-TC06</t>
+          <t>SPM-69-TC01
+SPM-69-TC04
+SPM-69-TC07
+SPM-69-TC09</t>
         </is>
       </c>
       <c r="F22" s="9" t="n"/>
     </row>
-    <row r="23" ht="71.5" customHeight="1">
+    <row r="23" ht="44.5" customHeight="1">
       <c r="A23" s="11" t="inlineStr">
         <is>
-          <t>AC7</t>
+          <t>AC6</t>
         </is>
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>Given the Event Coordinator changes an equipment requirement that already has a reservation, when the change is saved, then the requirement goes back to Technical Support Staff as Requested, showing the quantity already reserved, for them to review again; the reservation is not changed automatically and is not flagged.</t>
+          <t>The assigned Event Coordinator is notified when a reservation for their event is released or adjusted.</t>
         </is>
       </c>
       <c r="C23" s="8" t="n"/>
       <c r="D23" s="9" t="n"/>
       <c r="E23" s="11" t="inlineStr">
         <is>
-          <t>SPM-69-TC07
-SPM-69-TC08</t>
+          <t>SPM-69-TC02
+SPM-69-TC04
+SPM-69-TC07</t>
         </is>
       </c>
       <c r="F23" s="9" t="n"/>
     </row>
-    <row r="24" ht="31" customHeight="1">
+    <row r="24" ht="71.5" customHeight="1">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>AC8</t>
+          <t>AC7</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
         <is>
-          <t>A released reservation remains on the event record and is distinguishable from an active reservation.</t>
+          <t>Given the Event Coordinator changes an equipment requirement that already has a reservation, when the change is saved, then the requirement goes back to Technical Support Staff as Requested, showing the quantity already reserved, for them to review again; the reservation is not changed automatically and is not flagged.</t>
         </is>
       </c>
       <c r="C24" s="8" t="n"/>
       <c r="D24" s="9" t="n"/>
       <c r="E24" s="11" t="inlineStr">
         <is>
+          <t>SPM-69-TC03
+SPM-69-TC08
+SPM-69-TC09</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="n"/>
+    </row>
+    <row r="25" ht="31" customHeight="1">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>AC8</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>A released reservation remains on the event record and is distinguishable from an active reservation.</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="9" t="n"/>
+      <c r="E25" s="11" t="inlineStr">
+        <is>
           <t>SPM-69-TC01
 SPM-69-TC02</t>
         </is>
       </c>
-      <c r="F24" s="9" t="n"/>
-    </row>
-    <row r="26" ht="247" customHeight="1">
-      <c r="A26" s="7" t="inlineStr">
+      <c r="F25" s="9" t="n"/>
+    </row>
+    <row r="27" ht="247" customHeight="1">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>Code reviewed</t>
         </is>
       </c>
-      <c r="B26" s="11" t="inlineStr">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>src/app/api/events/[id]/equipment/[requestId]/reservation/route.ts
 src/lib/equipmentReservation.ts
@@ -1153,13 +1194,13 @@
 prisma/seed.ts</t>
         </is>
       </c>
-      <c r="C26" s="8" t="n"/>
-      <c r="D26" s="8" t="n"/>
-      <c r="E26" s="8" t="n"/>
-      <c r="F26" s="8" t="n"/>
-      <c r="G26" s="8" t="n"/>
-      <c r="H26" s="8" t="n"/>
-      <c r="I26" s="9" t="n"/>
+      <c r="C27" s="8" t="n"/>
+      <c r="D27" s="8" t="n"/>
+      <c r="E27" s="8" t="n"/>
+      <c r="F27" s="8" t="n"/>
+      <c r="G27" s="8" t="n"/>
+      <c r="H27" s="8" t="n"/>
+      <c r="I27" s="9" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="20">
@@ -1168,21 +1209,21 @@
     <mergeCell ref="B17:D17"/>
     <mergeCell ref="E23:F23"/>
     <mergeCell ref="E17:F17"/>
+    <mergeCell ref="B27:I27"/>
     <mergeCell ref="B19:D19"/>
     <mergeCell ref="E20:F20"/>
     <mergeCell ref="E19:F19"/>
     <mergeCell ref="B1:I1"/>
     <mergeCell ref="B24:D24"/>
     <mergeCell ref="B20:D20"/>
-    <mergeCell ref="B16:D16"/>
-    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="B25:D25"/>
+    <mergeCell ref="E25:F25"/>
     <mergeCell ref="B22:D22"/>
     <mergeCell ref="B18:D18"/>
     <mergeCell ref="E22:F22"/>
     <mergeCell ref="B21:D21"/>
     <mergeCell ref="E18:F18"/>
     <mergeCell ref="E21:F21"/>
-    <mergeCell ref="B26:I26"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId1"/>
@@ -1195,6 +1236,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1241,11 +1283,11 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Technical Support reviews a sent-back requirement and adjusts the reservation to the new quantity, marking it Reserved again</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="71.5" customHeight="1">
+          <t>A Coordinator's change to a reserved requirement sends it back to Technical Support as Requested, still showing what is reserved, without flagging it</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="98.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -1253,12 +1295,13 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>SPM-69-TC07 has just been run (SPM69 Coordinator Change Expo's Confidence Monitor line is back with Technical Support: 3 requested, 2 reserved, Status 'Requested'), and the tester is on its Equipment request page as Technical Support Staff.
-Data: run `npm run fixtures:spm69` after this case.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="44.5" customHeight="1">
+          <t>SPM69 Coordinator Change Expo (4 Jul 2028, Planning) has one line: Confidence Monitor, 2 requested, 2 reserved (Status 'Reserved'), technical requirements 'HDMI from the lectern'. Daniel Tan is its assigned Coordinator.
+Data: run `npm run fixtures:spm69` first. Go straight on to SPM-69-TC09, and run the script again after it.
+Logged out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="193" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1266,13 +1309,21 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>1. On the Confidence Monitor line, click 'Adjust'
-2. In 'Reserved quantity', enter 3
-3. Click 'Save'</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="17.5" customHeight="1">
+          <t>1. Log in as the Event Coordinator (daniel.tan@connectsphere.com, password123)
+2. Click 'All Events' in the sidebar
+3. Open the SPM69 Coordinator Change Expo event
+4. Click the 'Equipment' tab
+5. On the Confidence Monitor row, change 'Quantity' to 3
+6. Click 'Save'
+7. Click 'Flagged Arrangements' in the sidebar
+8. Click 'Log out'
+9. Log in as Technical Support Staff (vikram.nair@connectsphere.com, password123)
+10. Click 'Equipment Requests' in the sidebar
+11. Open the equipment request for the SPM69 Coordinator Change Expo event</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="31" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -1280,11 +1331,12 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Reserved quantity: 2 -&gt; 3 (the Coordinator's new quantity)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="71.5" customHeight="1">
+          <t>Event: SPM69 Coordinator Change Expo
+Quantity: 2 -&gt; 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="139" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1292,8 +1344,10 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 1: A form opens with 'Reserved quantity' showing 2.
-Step 3: The form closes and 'Reservation changed: 3 reserved.' appears on the line. Reserved shows 3, the Status chip shows 'Reserved', and 'The Coordinator changed this requirement' is no longer shown.</t>
+          <t>Step 4: The Confidence Monitor row shows the status 'Reserved' and '2 reserved'.
+Step 6: The row now shows the status 'Requested' and still '2 reserved'.
+Step 7: SPM69 Coordinator Change Expo is not listed.
+Step 11: The Confidence Monitor line shows Requested 3, Reserved 2 and Status 'Requested', with 'The Coordinator changed this requirement — 2 still reserved. Review it again.' and 'Technical requirements: HDMI from the lectern'. 'Adjust', 'Release' and 'Reserve' are offered.</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1468,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="31" customHeight="1">
+    <row r="3" ht="44.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Summary</t>
@@ -1422,11 +1476,11 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Adjust and Release are not offered on a line with nothing reserved, nor on a confirmed event</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="98.5" customHeight="1">
+          <t>Technical Support reviews a sent-back requirement and adjusts the reservation to the new quantity, marking it Reserved again</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="71.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -1434,13 +1488,12 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>SPM69 Overlap Seminar's Wireless Presenter line has nothing reserved (Status 'Requested'). SPM69 Confirmed Gala (11 Jul 2028, Confirmed) has 1 Mobile Charging Cart reserved.
-Data: run `npm run fixtures:spm69` first. This case changes nothing.
-Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="85" customHeight="1">
+          <t>SPM-69-TC08 has just been run (SPM69 Coordinator Change Expo's Confidence Monitor line is back with Technical Support: 3 requested, 2 reserved, Status 'Requested'), and the tester is on its Equipment request page as Technical Support Staff.
+Data: run `npm run fixtures:spm69` after this case.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1448,14 +1501,13 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'Equipment Requests' in the sidebar
-2. Open the equipment request for the SPM69 Overlap Seminar event
-3. Click 'Equipment Requests' in the breadcrumb
-4. Open the equipment request for the SPM69 Confirmed Gala event</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="31" customHeight="1">
+          <t>1. On the Confidence Monitor line, click 'Adjust'
+2. In 'Reserved quantity', enter 3
+3. Click 'Save'</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="17.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -1463,11 +1515,11 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Events: SPM69 Overlap Seminar (nothing reserved), SPM69 Confirmed Gala (Confirmed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="112" customHeight="1">
+          <t>Reserved quantity: 2 -&gt; 3 (the Coordinator's new quantity)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="71.5" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1475,8 +1527,8 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 2: The Wireless Presenter line shows Reserved '—' and Status 'Requested'. 'Reserve' and 'Update' are offered; 'Adjust' and 'Release' are not.
-Step 4: The page says 'This event is confirmed — its equipment is final. A change now goes through a change request.' The Mobile Charging Cart line shows Reserved 1 and Status 'Reserved', with no 'Adjust', 'Release', 'Reserve' or 'Update' button.</t>
+          <t>Step 1: A form opens with 'Reserved quantity' showing 2.
+Step 3: The form closes and 'Reservation changed: 3 reserved.' appears on the line. Reserved shows 3, the Status chip shows 'Reserved', and 'The Coordinator changed this requirement' is no longer shown.</t>
         </is>
       </c>
     </row>
@@ -1605,6 +1657,189 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
+          <t>Adjust and Release are not offered on a line with nothing reserved, nor on a confirmed event</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="98.5" customHeight="1">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>SPM69 Overlap Seminar's Wireless Presenter line has nothing reserved (Status 'Requested'). SPM69 Confirmed Gala (11 Jul 2028, Confirmed) has 1 Mobile Charging Cart reserved.
+Data: run `npm run fixtures:spm69` first. This case changes nothing.
+Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="85" customHeight="1">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Test Steps</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>1. Click 'Equipment Requests' in the sidebar
+2. Open the equipment request for the SPM69 Overlap Seminar event
+3. Click 'Equipment Requests' in the breadcrumb
+4. Open the equipment request for the SPM69 Confirmed Gala event</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="31" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Events: SPM69 Overlap Seminar (nothing reserved), SPM69 Confirmed Gala (Confirmed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="112" customHeight="1">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>Step 2: The Wireless Presenter line shows Reserved '—' and Status 'Requested'. 'Reserve' and 'Update' are offered; 'Adjust' and 'Release' are not.
+Step 4: The page says 'This event is confirmed — its equipment is final. A change now goes through a change request.' The Mobile Charging Cart line shows Reserved 1 and Status 'Reserved', with no 'Adjust', 'Release', 'Reserve' or 'Update' button.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17.5" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>kchoongg</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Creation Date</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>46317</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Date of Execution</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Commit</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <cols>
+    <col width="24.77734375" customWidth="1" min="1" max="1"/>
+    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17.5" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>SPM-69-TC11</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="31" customHeight="1">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
           <t>The Event Coordinator cannot release or adjust a reservation, even by typing the Equipment request page's address</t>
         </is>
       </c>
@@ -1756,7 +1991,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1814,60 +2049,82 @@
       </c>
       <c r="C4" s="11" t="n"/>
     </row>
-    <row r="5" ht="71.5" customHeight="1">
+    <row r="5" ht="98.5" customHeight="1">
       <c r="A5" s="11" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>DECIDED 2026-10-22 (kchoongg) - a requirement sent back by the Coordinator (AC7) keeps its reserved units counted against availability until Technical Support acts on it: adjusts, releases, reserves again, or marks it 'Cannot be provided'. That is how 'the reservation is not changed automatically' is built.</t>
+          <t>DECIDED 2026-10-26 (kchoongg) - a release needs a reason (required, up to 500 characters, the same cap as Technical notes). It is saved as Technical Support's notes, so both screens show it, and it is sent in the Coordinator's notification, so they can decide whether to remove the requirement or ask for the equipment again (TC01, TC02). Reserving a released line again clears the reason, as reserving clears a 'Cannot be provided' reason. Not in the story's wording.</t>
         </is>
       </c>
       <c r="C5" s="11" t="n"/>
     </row>
-    <row r="6" ht="139" customHeight="1">
+    <row r="6" ht="85" customHeight="1">
       <c r="A6" s="11" t="n">
         <v>5</v>
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>DECIDED 2026-10-22 (kchoongg) - screen wording, chosen to match the Reserve and Update panels: buttons 'Adjust' and 'Release'; field 'Reserved quantity'; dialog 'Release this reservation?'; confirmations 'Reservation changed: N reserved.' and 'Reservation released.'; refusals 'Only N available for this event's dates.', 'The event requested N — a reservation cannot be more than that.', 'Enter a whole number of at least 1. To free all of it, use Release.', 'That is already the reserved quantity.'; notifications 'Equipment reservation released' / 'Equipment reservation changed'; AC7 note 'The Coordinator changed this requirement — N still reserved. Review it again.'</t>
+          <t>DECIDED 2026-10-26 (kchoongg) - when the Coordinator changes the quantity of a released line, it goes back to Technical Support as a fresh request: Status 'Requested', nothing reserved, the release reason cleared (TC03). Changing only its technical requirements leaves it released, since that does not mean the event needs the equipment again. AC7 itself only covers lines that still have a reservation.</t>
         </is>
       </c>
       <c r="C6" s="11" t="n"/>
     </row>
-    <row r="7" ht="98.5" customHeight="1">
+    <row r="7" ht="71.5" customHeight="1">
       <c r="A7" s="11" t="n">
         <v>6</v>
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>OPEN - a released line still counts as an outstanding equipment arrangement when the Coordinator confirms the event or submits it for a safety check (only 'cancelled' lines are skipped in src/lib/eventConfirmation.ts and safetyCheck.ts). So after a release, the Coordinator must remove the requirement or mark it not required before confirming. This seems right, since the requirement is no longer met, but the team should confirm it.</t>
+          <t>DECIDED 2026-10-22 (kchoongg) - a requirement sent back by the Coordinator (AC7) keeps its reserved units counted against availability until Technical Support acts on it: adjusts, releases, reserves again, or marks it 'Cannot be provided'. That is how 'the reservation is not changed automatically' is built.</t>
         </is>
       </c>
       <c r="C7" s="11" t="n"/>
     </row>
-    <row r="8" ht="71.5" customHeight="1">
+    <row r="8" ht="166" customHeight="1">
       <c r="A8" s="11" t="n">
         <v>7</v>
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>OPEN - recording units out of service (SPM-55) flags only Reserved and Partially fulfilled lines whose reservation is now short. A line sent back to Technical Support (AC7) that still holds units is not flagged. Technical Support is reviewing that line anyway, so this was left as it is.</t>
+          <t>DECIDED 2026-10-22 (kchoongg) - screen wording, chosen to match the Reserve and Update panels: buttons 'Adjust' and 'Release'; field 'Reserved quantity'; dialog 'Release this reservation?' with a required 'Reason for releasing' field; confirmations 'Reservation changed: N reserved.' and 'Reservation released.'; refusals 'Only N available for this event's dates.', 'The event requested N — a reservation cannot be more than that.', 'Enter a whole number of at least 1. To free all of it, use Release.', 'That is already the reserved quantity.', 'Give a reason for releasing this reservation.', 'The reason must be 500 characters or fewer.'; notifications 'Equipment reservation released' / 'Equipment reservation changed'; AC7 note 'The Coordinator changed this requirement — N still reserved. Review it again.'</t>
         </is>
       </c>
       <c r="C8" s="11" t="n"/>
     </row>
-    <row r="9" ht="44.5" customHeight="1">
+    <row r="9" ht="98.5" customHeight="1">
       <c r="A9" s="11" t="n">
         <v>8</v>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
+          <t>OPEN - a released line still counts as an outstanding equipment arrangement when the Coordinator confirms the event or submits it for a safety check (only 'cancelled' lines are skipped in src/lib/eventConfirmation.ts and safetyCheck.ts). So after a release, the Coordinator must remove the requirement or mark it not required before confirming. This seems right, since the requirement is no longer met, but the team should confirm it.</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="n"/>
+    </row>
+    <row r="10" ht="71.5" customHeight="1">
+      <c r="A10" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>OPEN - recording units out of service (SPM-55) flags only Reserved and Partially fulfilled lines whose reservation is now short. A line sent back to Technical Support (AC7) that still holds units is not flagged. Technical Support is reviewing that line anyway, so this was left as it is.</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="n"/>
+    </row>
+    <row r="11" ht="44.5" customHeight="1">
+      <c r="A11" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
           <t>OPEN - no notification goes to Technical Support when a requirement comes back as Requested (AC7). The story only says it goes back to them; it shows on their Equipment request page with the note above.</t>
         </is>
       </c>
-      <c r="C9" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1915,7 +2172,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Technical Support releases a reservation after first cancelling, the line is marked Released, and its units become available to an overlapping event</t>
+          <t>Technical Support releases a reservation with a reason after first cancelling, the line is marked Released, and its units become available to an overlapping event</t>
         </is>
       </c>
     </row>
@@ -1935,7 +2192,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="179.5" customHeight="1">
+    <row r="5" ht="220" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -1950,13 +2207,15 @@
 5. On the Wireless Presenter line, click 'Release'
 6. In the dialog, click 'Cancel'
 7. On the Wireless Presenter line, click 'Release' again
-8. In the dialog, click 'Release'
-9. Click 'Equipment Requests' in the breadcrumb
-10. Open the equipment request for the SPM69 Overlap Seminar event</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="58" customHeight="1">
+8. In the dialog, click 'Release' without giving a reason
+9. In 'Reason for releasing', enter 'Client is bringing their own presenters'
+10. Click 'Release'
+11. Click 'Equipment Requests' in the breadcrumb
+12. Open the equipment request for the SPM69 Overlap Seminar event</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="71.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -1965,11 +2224,12 @@
       <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Released: SPM69 Release Rehearsal, Wireless Presenter (3 reserved)
+Reason: Client is bringing their own presenters
 Overlapping event: SPM69 Overlap Seminar, Wireless Presenter (3 requested)</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="287.5" customHeight="1">
+    <row r="7" ht="355" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -1979,10 +2239,11 @@
         <is>
           <t>Step 2: The Wireless Presenter line reads '4 total − 0 out of service − 3 reserved elsewhere = 1 available for these dates' and '3 requested, 1 available.' Its Availability chip shows 'Partial'.
 Step 4: The Wireless Presenter line shows Requested 3, Reserved 3 and Status 'Reserved', with 'Adjust' and 'Release' buttons and no 'Reserve' button.
-Step 5: A dialog 'Release this reservation?' appears, saying 'This frees the 3 Wireless Presenter reserved for SPM69 Release Rehearsal for other events. The event's Coordinator is told.'
+Step 5: A dialog 'Release this reservation?' appears, saying 'This frees the 3 Wireless Presenter reserved for SPM69 Release Rehearsal for other events. The event's Coordinator is told.', with an empty, required 'Reason for releasing' field.
 Step 6: The dialog closes. The line still shows Reserved 3 and Status 'Reserved'.
-Step 8: The dialog closes and 'Reservation released.' appears on the line. Its Status chip shows 'Released', the Reserved column shows '—', and the line says 'Released — 3 were reserved.' 'Adjust' and 'Release' are no longer offered; 'Reserve' is.
-Step 10: The Wireless Presenter line now reads '4 total − 0 out of service − 0 reserved elsewhere = 4 available for these dates' and its Availability chip shows 'Available'.</t>
+Step 8: 'Give a reason for releasing this reservation.' appears under 'Reason for releasing'. The dialog stays open and nothing is released.
+Step 10: The dialog closes and 'Reservation released.' appears on the line. Its Status chip shows 'Released', the Reserved column shows '—', the line says 'Released — 3 were reserved.' and 'Technical Support notes: Client is bringing their own presenters'. 'Adjust' and 'Release' are no longer offered; 'Reserve' is.
+Step 12: The Wireless Presenter line now reads '4 total − 0 out of service − 0 reserved elsewhere = 4 available for these dates' and its Availability chip shows 'Available'.</t>
         </is>
       </c>
     </row>
@@ -2111,11 +2372,11 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>The assigned Coordinator is notified of the release, and the released reservation stays on the event's Equipment tab marked Released</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="58" customHeight="1">
+          <t>The assigned Coordinator is notified of the release and its reason, and the released reservation stays on the event's Equipment tab marked Released</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="71.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2123,8 +2384,8 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>SPM-69-TC01 has just been run (the Wireless Presenter reservation of SPM69 Release Rehearsal was released). Daniel Tan is the event's assigned Coordinator.
-Data: run `npm run fixtures:spm69` after this case.</t>
+          <t>SPM-69-TC01 has just been run (the Wireless Presenter reservation of SPM69 Release Rehearsal was released, with a reason). Daniel Tan is the event's assigned Coordinator.
+Data: go straight on to SPM-69-TC03, and run `npm run fixtures:spm69` after it.</t>
         </is>
       </c>
     </row>
@@ -2156,7 +2417,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="85" customHeight="1">
+    <row r="7" ht="125.5" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2164,8 +2425,8 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 3: The list shows an unread notification 'Equipment reservation released' reading 'Technical Support released the 3 Wireless Presenter reserved for SPM69 Release Rehearsal.'
-Step 4: The Equipment tab of SPM69 Release Rehearsal opens. The Wireless Presenter row is still listed, with the status 'Released' and '3 released' beside it (not '3 reserved').</t>
+          <t>Step 3: The list shows an unread notification 'Equipment reservation released' reading 'Technical Support released the 3 Wireless Presenter reserved for SPM69 Release Rehearsal. Reason: Client is bringing their own presenters'
+Step 4: The Equipment tab of SPM69 Release Rehearsal opens. The Wireless Presenter row is still listed, with the status 'Released' and '3 released' beside it (not '3 reserved'), and 'Technical Support notes: Client is bringing their own presenters'.</t>
         </is>
       </c>
     </row>
@@ -2294,11 +2555,11 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Technical Support reduces a reservation, the line becomes Partially fulfilled, the freed units show as available to an overlapping event, and the Coordinator is notified</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="125.5" customHeight="1">
+          <t>Changing the quantity of a released line sends it back to Technical Support as a fresh request, while changing only its technical requirements leaves it released</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="58" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2306,15 +2567,12 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>Both events are on 20 Jun 2028 and use Confidence Monitor (4 in stock):
-- SPM69 Reduce Workshop: 4 requested, 4 reserved (Status 'Reserved')
-- SPM69 Neighbour Briefing: 2 requested, nothing reserved
-Data: run `npm run fixtures:spm69` before and after this case.
-Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="220" customHeight="1">
+          <t>SPM-69-TC02 has just been run: the Coordinator (Daniel Tan) is on the Equipment tab of SPM69 Release Rehearsal, whose Wireless Presenter line is Released (3 were reserved).
+Data: run `npm run fixtures:spm69` after this case.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="152.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2322,22 +2580,18 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>1. Click 'Equipment Requests' in the sidebar
-2. Open the equipment request for the SPM69 Neighbour Briefing event
-3. Click 'Equipment Requests' in the breadcrumb
-4. Open the equipment request for the SPM69 Reduce Workshop event
-5. On the Confidence Monitor line, click 'Adjust'
-6. In 'Reserved quantity', enter 2
-7. Click 'Save'
-8. Click 'Equipment Requests' in the breadcrumb
-9. Open the equipment request for the SPM69 Neighbour Briefing event
-10. Click 'Log out'
-11. Log in as the Event Coordinator (daniel.tan@connectsphere.com, password123)
-12. Click 'Notifications' in the sidebar</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="31" customHeight="1">
+          <t>1. On the Wireless Presenter row, change 'Technical requirements' to 'USB-C clicker'
+2. Click 'Save'
+3. On the Wireless Presenter row, change 'Quantity' to 2
+4. Click 'Save'
+5. Click 'Log out'
+6. Log in as Technical Support Staff (vikram.nair@connectsphere.com, password123)
+7. Click 'Equipment Requests' in the sidebar
+8. Open the equipment request for the SPM69 Release Rehearsal event</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -2345,12 +2599,13 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Event: SPM69 Reduce Workshop
-Reserved quantity: 4 -&gt; 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="220" customHeight="1">
+          <t>Event: SPM69 Release Rehearsal
+Technical requirements: 'USB-C clicker'
+Quantity: 3 -&gt; 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="139" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2358,11 +2613,9 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 2: The Confidence Monitor line reads '4 total − 0 out of service − 4 reserved elsewhere = 0 available for these dates' and 'Held by SPM69 Reduce Workshop (4 units) until 21 Jun.' Its Availability chip shows 'None available'.
-Step 5: A form opens on the line with a 'Reserved quantity' field showing 4, and 'Save' and 'Cancel' buttons.
-Step 7: The form closes and 'Reservation changed: 2 reserved.' appears on the line. Reserved shows 2 and the Status chip shows 'Partially fulfilled'.
-Step 9: The Confidence Monitor line now reads '4 total − 0 out of service − 2 reserved elsewhere = 2 available for these dates' and its Availability chip shows 'Available'.
-Step 12: The list shows an unread notification 'Equipment reservation changed' reading 'Technical Support changed the Confidence Monitor reserved for SPM69 Reduce Workshop from 4 to 2.'</t>
+          <t>Step 2: The row still shows the status 'Released' and '3 released'.
+Step 4: The row now shows the status 'Requested', with no reserved or released count beside it and no Technical Support notes.
+Step 8: The Wireless Presenter line shows Requested 2, Reserved '—' and Status 'Requested', with 'Technical requirements: USB-C clicker' and 'Technical Support notes: —'. It no longer says 'Released — 3 were reserved.' 'Reserve' is offered; 'Adjust' and 'Release' are not.</t>
         </is>
       </c>
     </row>
@@ -2483,7 +2736,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="31" customHeight="1">
+    <row r="3" ht="44.5" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Summary</t>
@@ -2491,11 +2744,11 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>An increase to one more unit than is available for the event's dates is refused and nothing is saved</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="152.5" customHeight="1">
+          <t>Technical Support reduces a reservation, the line becomes Partially fulfilled, the freed units show as available to an overlapping event, and the Coordinator is notified</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="125.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2503,16 +2756,15 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>Both events are on 27 Jun 2028 and use Wireless Presenter (4 in stock):
-- SPM69 Increase Forum: 4 requested, 2 reserved (Status 'Partially fulfilled')
-- SPM69 Rival Launch: 1 reserved
-So 3 are available to SPM69 Increase Forum (its own 2 are not counted against it).
-Data: run `npm run fixtures:spm69` first. This case changes nothing.
+          <t>Both events are on 20 Jun 2028 and use Confidence Monitor (4 in stock):
+- SPM69 Reduce Workshop: 4 requested, 4 reserved (Status 'Reserved')
+- SPM69 Neighbour Briefing: 2 requested, nothing reserved
+Data: run `npm run fixtures:spm69` before and after this case.
 Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="98.5" customHeight="1">
+    <row r="5" ht="220" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2521,15 +2773,21 @@
       <c r="B5" s="13" t="inlineStr">
         <is>
           <t>1. Click 'Equipment Requests' in the sidebar
-2. Open the equipment request for the SPM69 Increase Forum event
-3. On the Wireless Presenter line, click 'Adjust'
-4. In 'Reserved quantity', enter 4
-5. Click 'Save'
-6. Refresh the page</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="44.5" customHeight="1">
+2. Open the equipment request for the SPM69 Neighbour Briefing event
+3. Click 'Equipment Requests' in the breadcrumb
+4. Open the equipment request for the SPM69 Reduce Workshop event
+5. On the Confidence Monitor line, click 'Adjust'
+6. In 'Reserved quantity', enter 2
+7. Click 'Save'
+8. Click 'Equipment Requests' in the breadcrumb
+9. Open the equipment request for the SPM69 Neighbour Briefing event
+10. Click 'Log out'
+11. Log in as the Event Coordinator (daniel.tan@connectsphere.com, password123)
+12. Click 'Notifications' in the sidebar</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="31" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -2537,13 +2795,12 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Event: SPM69 Increase Forum
-Available: 3
-Reserved quantity: 2 -&gt; 4 (one more than available)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="112" customHeight="1">
+          <t>Event: SPM69 Reduce Workshop
+Reserved quantity: 4 -&gt; 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="220" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2551,9 +2808,11 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 2: The Wireless Presenter line reads '4 total − 0 out of service − 1 reserved elsewhere = 3 available for these dates', with Requested 4, Reserved 2 and Status 'Partially fulfilled'.
-Step 5: 'Only 3 available for this event's dates.' appears under 'Reserved quantity'. The form stays open.
-Step 6: The line still shows Reserved 2 and Status 'Partially fulfilled'.</t>
+          <t>Step 2: The Confidence Monitor line reads '4 total − 0 out of service − 4 reserved elsewhere = 0 available for these dates' and 'Held by SPM69 Reduce Workshop (4 units) until 21 Jun.' Its Availability chip shows 'None available'.
+Step 5: A form opens on the line with a 'Reserved quantity' field showing 4, and 'Save' and 'Cancel' buttons.
+Step 7: The form closes and 'Reservation changed: 2 reserved.' appears on the line. Reserved shows 2 and the Status chip shows 'Partially fulfilled'.
+Step 9: The Confidence Monitor line now reads '4 total − 0 out of service − 2 reserved elsewhere = 2 available for these dates' and its Availability chip shows 'Available'.
+Step 12: The list shows an unread notification 'Equipment reservation changed' reading 'Technical Support changed the Confidence Monitor reserved for SPM69 Reduce Workshop from 4 to 2.'</t>
         </is>
       </c>
     </row>
@@ -2682,11 +2941,11 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>The Adjust form refuses more than was requested, zero, and the quantity already reserved, and Cancel saves nothing</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="85" customHeight="1">
+          <t>An increase to one more unit than is available for the event's dates is refused and nothing is saved</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="152.5" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -2694,13 +2953,16 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>SPM69 Increase Forum's Wireless Presenter line: 4 requested, 2 reserved, 3 available (see SPM-69-TC04).
+          <t>Both events are on 27 Jun 2028 and use Wireless Presenter (4 in stock):
+- SPM69 Increase Forum: 4 requested, 2 reserved (Status 'Partially fulfilled')
+- SPM69 Rival Launch: 1 reserved
+So 3 are available to SPM69 Increase Forum (its own 2 are not counted against it).
 Data: run `npm run fixtures:spm69` first. This case changes nothing.
 Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="152.5" customHeight="1">
+    <row r="5" ht="98.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2711,17 +2973,13 @@
           <t>1. Click 'Equipment Requests' in the sidebar
 2. Open the equipment request for the SPM69 Increase Forum event
 3. On the Wireless Presenter line, click 'Adjust'
-4. In 'Reserved quantity', enter 5
+4. In 'Reserved quantity', enter 4
 5. Click 'Save'
-6. In 'Reserved quantity', enter 0
-7. Click 'Save'
-8. In 'Reserved quantity', enter 2
-9. Click 'Save'
-10. Click 'Cancel'</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="31" customHeight="1">
+6. Refresh the page</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="44.5" customHeight="1">
       <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Test Data</t>
@@ -2729,11 +2987,13 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Reserved quantity: 5 (more than the 4 requested), 0, 2 (unchanged)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="125.5" customHeight="1">
+          <t>Event: SPM69 Increase Forum
+Available: 3
+Reserved quantity: 2 -&gt; 4 (one more than available)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="112" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -2741,10 +3001,9 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 5: 'The event requested 4 — a reservation cannot be more than that.' appears under 'Reserved quantity'.
-Step 7: 'Enter a whole number of at least 1. To free all of it, use Release.' appears under 'Reserved quantity'.
-Step 9: 'That is already the reserved quantity.' appears under 'Reserved quantity'.
-Step 10: The form closes. The line still shows Reserved 2 and Status 'Partially fulfilled', with no confirmation message.</t>
+          <t>Step 2: The Wireless Presenter line reads '4 total − 0 out of service − 1 reserved elsewhere = 3 available for these dates', with Requested 4, Reserved 2 and Status 'Partially fulfilled'.
+Step 5: 'Only 3 available for this event's dates.' appears under 'Reserved quantity'. The form stays open.
+Step 6: The line still shows Reserved 2 and Status 'Partially fulfilled'.</t>
         </is>
       </c>
     </row>
@@ -2873,7 +3132,7 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Technical Support increases a reservation to exactly what is available, and the Coordinator is notified</t>
+          <t>The Adjust form refuses more than was requested, zero, and the quantity already reserved, and Cancel saves nothing</t>
         </is>
       </c>
     </row>
@@ -2885,13 +3144,13 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>SPM69 Increase Forum's Wireless Presenter line: 4 requested, 2 reserved, 3 available (see SPM-69-TC04).
-Data: run `npm run fixtures:spm69` before and after this case.
+          <t>SPM69 Increase Forum's Wireless Presenter line: 4 requested, 2 reserved, 3 available (see SPM-69-TC05).
+Data: run `npm run fixtures:spm69` first. This case changes nothing.
 Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="139" customHeight="1">
+    <row r="5" ht="152.5" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -2902,11 +3161,13 @@
           <t>1. Click 'Equipment Requests' in the sidebar
 2. Open the equipment request for the SPM69 Increase Forum event
 3. On the Wireless Presenter line, click 'Adjust'
-4. In 'Reserved quantity', enter 3
+4. In 'Reserved quantity', enter 5
 5. Click 'Save'
-6. Click 'Log out'
-7. Log in as the Event Coordinator (daniel.tan@connectsphere.com, password123)
-8. Click 'Notifications' in the sidebar</t>
+6. In 'Reserved quantity', enter 0
+7. Click 'Save'
+8. In 'Reserved quantity', enter 2
+9. Click 'Save'
+10. Click 'Cancel'</t>
         </is>
       </c>
     </row>
@@ -2918,8 +3179,7 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Event: SPM69 Increase Forum
-Reserved quantity: 2 -&gt; 3 (exactly what is available)</t>
+          <t>Reserved quantity: 5 (more than the 4 requested), 0, 2 (unchanged)</t>
         </is>
       </c>
     </row>
@@ -2931,8 +3191,10 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 5: The form closes and 'Reservation changed: 3 reserved.' appears on the line. Reserved shows 3 and the Status chip stays 'Partially fulfilled' (3 of the 4 requested). The line still reads '4 total − 0 out of service − 1 reserved elsewhere = 3 available for these dates'.
-Step 8: The list shows an unread notification 'Equipment reservation changed' reading 'Technical Support changed the Wireless Presenter reserved for SPM69 Increase Forum from 2 to 3.'</t>
+          <t>Step 5: 'The event requested 4 — a reservation cannot be more than that.' appears under 'Reserved quantity'.
+Step 7: 'Enter a whole number of at least 1. To free all of it, use Release.' appears under 'Reserved quantity'.
+Step 9: 'That is already the reserved quantity.' appears under 'Reserved quantity'.
+Step 10: The form closes. The line still shows Reserved 2 and Status 'Partially fulfilled', with no confirmation message.</t>
         </is>
       </c>
     </row>
@@ -3053,7 +3315,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="44.5" customHeight="1">
+    <row r="3" ht="31" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Summary</t>
@@ -3061,11 +3323,11 @@
       </c>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>A Coordinator's change to a reserved requirement sends it back to Technical Support as Requested, still showing what is reserved, without flagging it</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="98.5" customHeight="1">
+          <t>Technical Support increases a reservation to exactly what is available, and the Coordinator is notified</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="85" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
@@ -3073,13 +3335,13 @@
       </c>
       <c r="B4" s="13" t="inlineStr">
         <is>
-          <t>SPM69 Coordinator Change Expo (4 Jul 2028, Planning) has one line: Confidence Monitor, 2 requested, 2 reserved (Status 'Reserved'), technical requirements 'HDMI from the lectern'. Daniel Tan is its assigned Coordinator.
-Data: run `npm run fixtures:spm69` first. Go straight on to SPM-69-TC08, and run the script again after it.
-Logged out.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="193" customHeight="1">
+          <t>SPM69 Increase Forum's Wireless Presenter line: 4 requested, 2 reserved, 3 available (see SPM-69-TC05).
+Data: run `npm run fixtures:spm69` before and after this case.
+Logged in as Technical Support Staff (vikram.nair@connectsphere.com, password123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="139" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Test Steps</t>
@@ -3087,17 +3349,14 @@
       </c>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>1. Log in as the Event Coordinator (daniel.tan@connectsphere.com, password123)
-2. Click 'All Events' in the sidebar
-3. Open the SPM69 Coordinator Change Expo event
-4. Click the 'Equipment' tab
-5. On the Confidence Monitor row, change 'Quantity' to 3
-6. Click 'Save'
-7. Click 'Flagged Arrangements' in the sidebar
-8. Click 'Log out'
-9. Log in as Technical Support Staff (vikram.nair@connectsphere.com, password123)
-10. Click 'Equipment Requests' in the sidebar
-11. Open the equipment request for the SPM69 Coordinator Change Expo event</t>
+          <t>1. Click 'Equipment Requests' in the sidebar
+2. Open the equipment request for the SPM69 Increase Forum event
+3. On the Wireless Presenter line, click 'Adjust'
+4. In 'Reserved quantity', enter 3
+5. Click 'Save'
+6. Click 'Log out'
+7. Log in as the Event Coordinator (daniel.tan@connectsphere.com, password123)
+8. Click 'Notifications' in the sidebar</t>
         </is>
       </c>
     </row>
@@ -3109,12 +3368,12 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Event: SPM69 Coordinator Change Expo
-Quantity: 2 -&gt; 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="139" customHeight="1">
+          <t>Event: SPM69 Increase Forum
+Reserved quantity: 2 -&gt; 3 (exactly what is available)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="125.5" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Expected Result</t>
@@ -3122,10 +3381,8 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Step 4: The Confidence Monitor row shows the status 'Reserved' and '2 reserved'.
-Step 6: The row now shows the status 'Requested' and still '2 reserved'.
-Step 7: SPM69 Coordinator Change Expo is not listed.
-Step 11: The Confidence Monitor line shows Requested 3, Reserved 2 and Status 'Requested', with 'The Coordinator changed this requirement — 2 still reserved. Review it again.' and 'Technical requirements: HDMI from the lectern'. 'Adjust', 'Release' and 'Reserve' are offered.</t>
+          <t>Step 5: The form closes and 'Reservation changed: 3 reserved.' appears on the line. Reserved shows 3 and the Status chip stays 'Partially fulfilled' (3 of the 4 requested). The line still reads '4 total − 0 out of service − 1 reserved elsewhere = 3 available for these dates'.
+Step 8: The list shows an unread notification 'Equipment reservation changed' reading 'Technical Support changed the Wireless Presenter reserved for SPM69 Increase Forum from 2 to 3.'</t>
         </is>
       </c>
     </row>

</xml_diff>